<commit_message>
Introduced Dynamic Scopus Data Download
</commit_message>
<xml_diff>
--- a/output/cfr_scopus_scimago_results.xlsx
+++ b/output/cfr_scopus_scimago_results.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="n">
-        <v>1.45</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="3">
@@ -737,7 +737,7 @@
       </c>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="n">
-        <v>1.31</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="4">
@@ -839,7 +839,7 @@
       </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="n">
-        <v>2.2</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="5">
@@ -941,7 +941,7 @@
       </c>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="n">
-        <v>1.71</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="6">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="n">
-        <v>2.35</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="7">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="n">
-        <v>1.44</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="8">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="n">
-        <v>1.96</v>
+        <v>1.67</v>
       </c>
     </row>
     <row r="9">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="n">
-        <v>1.8</v>
+        <v>2.11</v>
       </c>
     </row>
     <row r="10">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="n">
-        <v>2.32</v>
+        <v>3.67</v>
       </c>
     </row>
     <row r="11">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>2.29</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="12">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="n">
-        <v>1.05</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="13">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="n">
-        <v>1.11</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="14">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="n">
-        <v>1.21</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="15">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="n">
-        <v>1.57</v>
+        <v>1.01</v>
       </c>
     </row>
     <row r="16">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="n">
-        <v>2.5</v>
+        <v>1.27</v>
       </c>
     </row>
     <row r="17">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="n">
-        <v>1.12</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="18">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="n">
-        <v>1.93</v>
+        <v>1.06</v>
       </c>
     </row>
     <row r="19">
@@ -2393,7 +2393,7 @@
       </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>11.49</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="20">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="n">
-        <v>1.79</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="21">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>13.6</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="22">
@@ -2711,7 +2711,7 @@
       </c>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="n">
-        <v>4.24</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="23">
@@ -2817,7 +2817,7 @@
       </c>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>34.7</v>
+        <v>1.61</v>
       </c>
     </row>
     <row r="24">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>33.56</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="25">
@@ -3029,7 +3029,7 @@
       </c>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="n">
-        <v>10.94</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="26">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="n">
-        <v>1.42</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="27">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="n">
-        <v>2.95</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="28">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="n">
-        <v>5.88</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="29">
@@ -3445,7 +3445,7 @@
       </c>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="n">
-        <v>3.46</v>
+        <v>2.31</v>
       </c>
     </row>
     <row r="30">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="U30" t="inlineStr"/>
       <c r="V30" t="n">
-        <v>7.3</v>
+        <v>4.31</v>
       </c>
     </row>
     <row r="31">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="U31" t="inlineStr"/>
       <c r="V31" t="n">
-        <v>2.04</v>
+        <v>2.52</v>
       </c>
     </row>
     <row r="32">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="U32" t="inlineStr"/>
       <c r="V32" t="n">
-        <v>2.37</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="33">
@@ -3865,7 +3865,7 @@
       </c>
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="n">
-        <v>2.85</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="34">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="U34" t="inlineStr"/>
       <c r="V34" t="n">
-        <v>1.49</v>
+        <v>1.97</v>
       </c>
     </row>
     <row r="35">
@@ -4073,7 +4073,7 @@
       </c>
       <c r="U35" t="inlineStr"/>
       <c r="V35" t="n">
-        <v>4.83</v>
+        <v>3.47</v>
       </c>
     </row>
     <row r="36">
@@ -4179,7 +4179,7 @@
       </c>
       <c r="U36" t="inlineStr"/>
       <c r="V36" t="n">
-        <v>18.33</v>
+        <v>9.01</v>
       </c>
     </row>
     <row r="37">
@@ -4281,7 +4281,7 @@
       </c>
       <c r="U37" t="inlineStr"/>
       <c r="V37" t="n">
-        <v>3.92</v>
+        <v>2.64</v>
       </c>
     </row>
     <row r="38">
@@ -4387,7 +4387,7 @@
       </c>
       <c r="U38" t="inlineStr"/>
       <c r="V38" t="n">
-        <v>5.9</v>
+        <v>3.38</v>
       </c>
     </row>
     <row r="39">
@@ -4493,7 +4493,7 @@
       </c>
       <c r="U39" t="inlineStr"/>
       <c r="V39" t="n">
-        <v>6.4</v>
+        <v>9.460000000000001</v>
       </c>
     </row>
     <row r="40">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="U40" t="inlineStr"/>
       <c r="V40" t="n">
-        <v>1.32</v>
+        <v>9.529999999999999</v>
       </c>
     </row>
     <row r="41">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="U41" t="inlineStr"/>
       <c r="V41" t="n">
-        <v>1.19</v>
+        <v>9.19</v>
       </c>
     </row>
     <row r="42">
@@ -4803,7 +4803,7 @@
       </c>
       <c r="U42" t="inlineStr"/>
       <c r="V42" t="n">
-        <v>1.24</v>
+        <v>8.67</v>
       </c>
     </row>
     <row r="43">
@@ -4909,7 +4909,7 @@
       </c>
       <c r="U43" t="inlineStr"/>
       <c r="V43" t="n">
-        <v>1.98</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="44">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="U44" t="inlineStr"/>
       <c r="V44" t="n">
-        <v>1.56</v>
+        <v>2.43</v>
       </c>
     </row>
     <row r="45">
@@ -5117,7 +5117,7 @@
       </c>
       <c r="U45" t="inlineStr"/>
       <c r="V45" t="n">
-        <v>1.45</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="46">
@@ -5223,7 +5223,7 @@
       </c>
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="n">
-        <v>2.66</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="47">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="U47" t="inlineStr"/>
       <c r="V47" t="n">
-        <v>2.61</v>
+        <v>1.54</v>
       </c>
     </row>
     <row r="48">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="U48" t="inlineStr"/>
       <c r="V48" t="n">
-        <v>2.98</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="49">
@@ -5541,7 +5541,7 @@
       </c>
       <c r="U49" t="inlineStr"/>
       <c r="V49" t="n">
-        <v>2.34</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="50">
@@ -5647,7 +5647,7 @@
       </c>
       <c r="U50" t="inlineStr"/>
       <c r="V50" t="n">
-        <v>2.05</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="51">
@@ -5753,7 +5753,7 @@
       </c>
       <c r="U51" t="inlineStr"/>
       <c r="V51" t="n">
-        <v>1.41</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="52">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="U52" t="inlineStr"/>
       <c r="V52" t="n">
-        <v>1.23</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="53">
@@ -5965,7 +5965,7 @@
       </c>
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="n">
-        <v>1.17</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="54">
@@ -6067,7 +6067,7 @@
       </c>
       <c r="U54" t="inlineStr"/>
       <c r="V54" t="n">
-        <v>1.22</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="55">
@@ -6173,7 +6173,7 @@
       </c>
       <c r="U55" t="inlineStr"/>
       <c r="V55" t="n">
-        <v>0.99</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="56">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="U56" t="inlineStr"/>
       <c r="V56" t="n">
-        <v>1.56</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="57">
@@ -6381,7 +6381,7 @@
       </c>
       <c r="U57" t="inlineStr"/>
       <c r="V57" t="n">
-        <v>2.08</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="58">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="U58" t="inlineStr"/>
       <c r="V58" t="n">
-        <v>1.27</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="59">
@@ -6589,7 +6589,7 @@
       </c>
       <c r="U59" t="inlineStr"/>
       <c r="V59" t="n">
-        <v>1.71</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="60">
@@ -6695,7 +6695,7 @@
       </c>
       <c r="U60" t="inlineStr"/>
       <c r="V60" t="n">
-        <v>1.6</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="61">
@@ -6797,7 +6797,7 @@
       </c>
       <c r="U61" t="inlineStr"/>
       <c r="V61" t="n">
-        <v>1.53</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="62">
@@ -6899,7 +6899,7 @@
       </c>
       <c r="U62" t="inlineStr"/>
       <c r="V62" t="n">
-        <v>3.07</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="63">
@@ -7005,7 +7005,7 @@
       </c>
       <c r="U63" t="inlineStr"/>
       <c r="V63" t="n">
-        <v>1.1</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="64">
@@ -7111,7 +7111,7 @@
       </c>
       <c r="U64" t="inlineStr"/>
       <c r="V64" t="n">
-        <v>0.96</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="65">
@@ -7217,7 +7217,7 @@
       </c>
       <c r="U65" t="inlineStr"/>
       <c r="V65" t="n">
-        <v>1.3</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="66">
@@ -7323,7 +7323,7 @@
       </c>
       <c r="U66" t="inlineStr"/>
       <c r="V66" t="n">
-        <v>1.17</v>
+        <v>1.51</v>
       </c>
     </row>
     <row r="67">
@@ -7425,7 +7425,7 @@
       </c>
       <c r="U67" t="inlineStr"/>
       <c r="V67" t="n">
-        <v>1.39</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="68">
@@ -7531,7 +7531,7 @@
       </c>
       <c r="U68" t="inlineStr"/>
       <c r="V68" t="n">
-        <v>1.11</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="69">
@@ -7637,7 +7637,7 @@
       </c>
       <c r="U69" t="inlineStr"/>
       <c r="V69" t="n">
-        <v>1.83</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="70">
@@ -7743,7 +7743,7 @@
       </c>
       <c r="U70" t="inlineStr"/>
       <c r="V70" t="n">
-        <v>1.21</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="71">
@@ -7845,7 +7845,7 @@
       </c>
       <c r="U71" t="inlineStr"/>
       <c r="V71" t="n">
-        <v>1.11</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="72">
@@ -7951,7 +7951,7 @@
       </c>
       <c r="U72" t="inlineStr"/>
       <c r="V72" t="n">
-        <v>1.06</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="73">
@@ -8057,7 +8057,7 @@
       </c>
       <c r="U73" t="inlineStr"/>
       <c r="V73" t="n">
-        <v>1.54</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="74">
@@ -8163,7 +8163,7 @@
       </c>
       <c r="U74" t="inlineStr"/>
       <c r="V74" t="n">
-        <v>1.18</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="75">
@@ -8269,7 +8269,7 @@
       </c>
       <c r="U75" t="inlineStr"/>
       <c r="V75" t="n">
-        <v>2.02</v>
+        <v>2.38</v>
       </c>
     </row>
     <row r="76">
@@ -8371,7 +8371,7 @@
       </c>
       <c r="U76" t="inlineStr"/>
       <c r="V76" t="n">
-        <v>1.45</v>
+        <v>2.69</v>
       </c>
     </row>
     <row r="77">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="U77" t="inlineStr"/>
       <c r="V77" t="n">
-        <v>1.32</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="78">
@@ -8579,7 +8579,7 @@
       </c>
       <c r="U78" t="inlineStr"/>
       <c r="V78" t="n">
-        <v>2.06</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="79">
@@ -8685,7 +8685,7 @@
       </c>
       <c r="U79" t="inlineStr"/>
       <c r="V79" t="n">
-        <v>1.24</v>
+        <v>2.81</v>
       </c>
     </row>
     <row r="80">
@@ -8791,7 +8791,7 @@
       </c>
       <c r="U80" t="inlineStr"/>
       <c r="V80" t="n">
-        <v>2</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="81">
@@ -8897,7 +8897,7 @@
       </c>
       <c r="U81" t="inlineStr"/>
       <c r="V81" t="n">
-        <v>1.37</v>
+        <v>2.43</v>
       </c>
     </row>
     <row r="82">
@@ -9003,7 +9003,7 @@
       </c>
       <c r="U82" t="inlineStr"/>
       <c r="V82" t="n">
-        <v>1.07</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="83">
@@ -9109,7 +9109,7 @@
       </c>
       <c r="U83" t="inlineStr"/>
       <c r="V83" t="n">
-        <v>1.87</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="84">
@@ -9215,7 +9215,7 @@
       </c>
       <c r="U84" t="inlineStr"/>
       <c r="V84" t="n">
-        <v>1.08</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="85">
@@ -9321,7 +9321,7 @@
       </c>
       <c r="U85" t="inlineStr"/>
       <c r="V85" t="n">
-        <v>1.36</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="86">
@@ -9423,7 +9423,7 @@
       </c>
       <c r="U86" t="inlineStr"/>
       <c r="V86" t="n">
-        <v>1.63</v>
+        <v>3.95</v>
       </c>
     </row>
     <row r="87">
@@ -9529,7 +9529,7 @@
       </c>
       <c r="U87" t="inlineStr"/>
       <c r="V87" t="n">
-        <v>1.03</v>
+        <v>5.45</v>
       </c>
     </row>
     <row r="88">
@@ -9635,7 +9635,7 @@
       </c>
       <c r="U88" t="inlineStr"/>
       <c r="V88" t="n">
-        <v>1.62</v>
+        <v>3.95</v>
       </c>
     </row>
     <row r="89">
@@ -9737,7 +9737,7 @@
       </c>
       <c r="U89" t="inlineStr"/>
       <c r="V89" t="n">
-        <v>1.29</v>
+        <v>4.01</v>
       </c>
     </row>
     <row r="90">
@@ -9839,7 +9839,7 @@
       </c>
       <c r="U90" t="inlineStr"/>
       <c r="V90" t="n">
-        <v>1.41</v>
+        <v>4.45</v>
       </c>
     </row>
     <row r="91">
@@ -9941,7 +9941,7 @@
       </c>
       <c r="U91" t="inlineStr"/>
       <c r="V91" t="n">
-        <v>1.65</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="92">
@@ -10047,7 +10047,7 @@
       </c>
       <c r="U92" t="inlineStr"/>
       <c r="V92" t="n">
-        <v>1.82</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="93">
@@ -10153,7 +10153,7 @@
       </c>
       <c r="U93" t="inlineStr"/>
       <c r="V93" t="n">
-        <v>1.02</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="94">
@@ -10255,7 +10255,7 @@
       </c>
       <c r="U94" t="inlineStr"/>
       <c r="V94" t="n">
-        <v>1.82</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="95">
@@ -10361,7 +10361,7 @@
       </c>
       <c r="U95" t="inlineStr"/>
       <c r="V95" t="n">
-        <v>1.4</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="96">
@@ -10467,7 +10467,7 @@
       </c>
       <c r="U96" t="inlineStr"/>
       <c r="V96" t="n">
-        <v>1.23</v>
+        <v>2.28</v>
       </c>
     </row>
     <row r="97">
@@ -10573,7 +10573,7 @@
       </c>
       <c r="U97" t="inlineStr"/>
       <c r="V97" t="n">
-        <v>1.56</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="98">
@@ -10679,7 +10679,7 @@
       </c>
       <c r="U98" t="inlineStr"/>
       <c r="V98" t="n">
-        <v>1.4</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="99">
@@ -10785,7 +10785,7 @@
       </c>
       <c r="U99" t="inlineStr"/>
       <c r="V99" t="n">
-        <v>1.11</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="100">
@@ -10891,7 +10891,7 @@
       </c>
       <c r="U100" t="inlineStr"/>
       <c r="V100" t="n">
-        <v>1.5</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="101">
@@ -10997,7 +10997,7 @@
       </c>
       <c r="U101" t="inlineStr"/>
       <c r="V101" t="n">
-        <v>1.28</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="102">
@@ -11103,7 +11103,7 @@
       </c>
       <c r="U102" t="inlineStr"/>
       <c r="V102" t="n">
-        <v>1.28</v>
+        <v>1.96</v>
       </c>
     </row>
     <row r="103">
@@ -11209,7 +11209,7 @@
       </c>
       <c r="U103" t="inlineStr"/>
       <c r="V103" t="n">
-        <v>0.96</v>
+        <v>3.67</v>
       </c>
     </row>
     <row r="104">
@@ -11315,7 +11315,7 @@
       </c>
       <c r="U104" t="inlineStr"/>
       <c r="V104" t="n">
-        <v>1.64</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="105">
@@ -11421,7 +11421,7 @@
       </c>
       <c r="U105" t="inlineStr"/>
       <c r="V105" t="n">
-        <v>1.19</v>
+        <v>3.14</v>
       </c>
     </row>
     <row r="106">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="U106" t="inlineStr"/>
       <c r="V106" t="n">
-        <v>1.16</v>
+        <v>3.17</v>
       </c>
     </row>
     <row r="107">
@@ -11629,7 +11629,7 @@
       </c>
       <c r="U107" t="inlineStr"/>
       <c r="V107" t="n">
-        <v>1.59</v>
+        <v>2.83</v>
       </c>
     </row>
     <row r="108">
@@ -11735,7 +11735,7 @@
       </c>
       <c r="U108" t="inlineStr"/>
       <c r="V108" t="n">
-        <v>1.52</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="109">
@@ -11841,7 +11841,7 @@
       </c>
       <c r="U109" t="inlineStr"/>
       <c r="V109" t="n">
-        <v>1.26</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="110">
@@ -11947,7 +11947,7 @@
       </c>
       <c r="U110" t="inlineStr"/>
       <c r="V110" t="n">
-        <v>1.96</v>
+        <v>2.58</v>
       </c>
     </row>
     <row r="111">
@@ -12049,7 +12049,7 @@
       </c>
       <c r="U111" t="inlineStr"/>
       <c r="V111" t="n">
-        <v>2.31</v>
+        <v>2.23</v>
       </c>
     </row>
     <row r="112">
@@ -12155,7 +12155,7 @@
       </c>
       <c r="U112" t="inlineStr"/>
       <c r="V112" t="n">
-        <v>1.04</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="113">
@@ -12261,7 +12261,7 @@
       </c>
       <c r="U113" t="inlineStr"/>
       <c r="V113" t="n">
-        <v>1.2</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="114">
@@ -12367,7 +12367,7 @@
       </c>
       <c r="U114" t="inlineStr"/>
       <c r="V114" t="n">
-        <v>1.33</v>
+        <v>2.32</v>
       </c>
     </row>
     <row r="115">
@@ -12473,7 +12473,7 @@
       </c>
       <c r="U115" t="inlineStr"/>
       <c r="V115" t="n">
-        <v>1.22</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="116">
@@ -12579,7 +12579,7 @@
       </c>
       <c r="U116" t="inlineStr"/>
       <c r="V116" t="n">
-        <v>1.96</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="117">
@@ -12685,7 +12685,7 @@
       </c>
       <c r="U117" t="inlineStr"/>
       <c r="V117" t="n">
-        <v>1.71</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="118">
@@ -12791,7 +12791,7 @@
       </c>
       <c r="U118" t="inlineStr"/>
       <c r="V118" t="n">
-        <v>1.49</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="119">
@@ -12999,7 +12999,7 @@
       </c>
       <c r="U120" t="inlineStr"/>
       <c r="V120" t="n">
-        <v>1.58</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="121">
@@ -13105,7 +13105,7 @@
       </c>
       <c r="U121" t="inlineStr"/>
       <c r="V121" t="n">
-        <v>1.46</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="122">
@@ -13211,7 +13211,7 @@
       </c>
       <c r="U122" t="inlineStr"/>
       <c r="V122" t="n">
-        <v>1.09</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="123">
@@ -13317,7 +13317,7 @@
       </c>
       <c r="U123" t="inlineStr"/>
       <c r="V123" t="n">
-        <v>1.74</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="124">
@@ -13423,7 +13423,7 @@
       </c>
       <c r="U124" t="inlineStr"/>
       <c r="V124" t="n">
-        <v>1.21</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="125">
@@ -13525,7 +13525,7 @@
       </c>
       <c r="U125" t="inlineStr"/>
       <c r="V125" t="n">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="126">
@@ -13631,7 +13631,7 @@
       </c>
       <c r="U126" t="inlineStr"/>
       <c r="V126" t="n">
-        <v>1.57</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="127">
@@ -13737,7 +13737,7 @@
       </c>
       <c r="U127" t="inlineStr"/>
       <c r="V127" t="n">
-        <v>1.78</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="128">
@@ -13843,7 +13843,7 @@
       </c>
       <c r="U128" t="inlineStr"/>
       <c r="V128" t="n">
-        <v>1.32</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="129">
@@ -13945,7 +13945,7 @@
       </c>
       <c r="U129" t="inlineStr"/>
       <c r="V129" t="n">
-        <v>1.67</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="130">
@@ -14047,7 +14047,7 @@
       </c>
       <c r="U130" t="inlineStr"/>
       <c r="V130" t="n">
-        <v>1.37</v>
+        <v>1.45</v>
       </c>
     </row>
     <row r="131">
@@ -14149,7 +14149,7 @@
       </c>
       <c r="U131" t="inlineStr"/>
       <c r="V131" t="n">
-        <v>1.48</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="132">
@@ -14255,7 +14255,7 @@
       </c>
       <c r="U132" t="inlineStr"/>
       <c r="V132" t="n">
-        <v>1.4</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="133">
@@ -14357,7 +14357,7 @@
       </c>
       <c r="U133" t="inlineStr"/>
       <c r="V133" t="n">
-        <v>1.56</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="134">
@@ -14459,7 +14459,7 @@
       </c>
       <c r="U134" t="inlineStr"/>
       <c r="V134" t="n">
-        <v>1.97</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="135">
@@ -14561,7 +14561,7 @@
       </c>
       <c r="U135" t="inlineStr"/>
       <c r="V135" t="n">
-        <v>1.75</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="136">
@@ -14663,7 +14663,7 @@
       </c>
       <c r="U136" t="inlineStr"/>
       <c r="V136" t="n">
-        <v>1.52</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="137">
@@ -14769,7 +14769,7 @@
       </c>
       <c r="U137" t="inlineStr"/>
       <c r="V137" t="n">
-        <v>1.84</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="138">
@@ -14875,7 +14875,7 @@
       </c>
       <c r="U138" t="inlineStr"/>
       <c r="V138" t="n">
-        <v>1.41</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="139">
@@ -14977,7 +14977,7 @@
       </c>
       <c r="U139" t="inlineStr"/>
       <c r="V139" t="n">
-        <v>1.04</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="140">
@@ -15083,7 +15083,7 @@
       </c>
       <c r="U140" t="inlineStr"/>
       <c r="V140" t="n">
-        <v>1.39</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="141">
@@ -15189,7 +15189,7 @@
       </c>
       <c r="U141" t="inlineStr"/>
       <c r="V141" t="n">
-        <v>1.73</v>
+        <v>1.44</v>
       </c>
     </row>
     <row r="142">
@@ -15295,7 +15295,7 @@
       </c>
       <c r="U142" t="inlineStr"/>
       <c r="V142" t="n">
-        <v>4.58</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="143">
@@ -15401,7 +15401,7 @@
       </c>
       <c r="U143" t="inlineStr"/>
       <c r="V143" t="n">
-        <v>3</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="144">
@@ -15503,7 +15503,7 @@
       </c>
       <c r="U144" t="inlineStr"/>
       <c r="V144" t="n">
-        <v>1.68</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="145">
@@ -15609,7 +15609,7 @@
       </c>
       <c r="U145" t="inlineStr"/>
       <c r="V145" t="n">
-        <v>1.73</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="146">
@@ -15711,7 +15711,7 @@
       </c>
       <c r="U146" t="inlineStr"/>
       <c r="V146" t="n">
-        <v>1.62</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="147">
@@ -15817,7 +15817,7 @@
       </c>
       <c r="U147" t="inlineStr"/>
       <c r="V147" t="n">
-        <v>1.49</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="148">
@@ -15923,7 +15923,7 @@
       </c>
       <c r="U148" t="inlineStr"/>
       <c r="V148" t="n">
-        <v>1.43</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="149">
@@ -16025,7 +16025,7 @@
       </c>
       <c r="U149" t="inlineStr"/>
       <c r="V149" t="n">
-        <v>1.67</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="150">
@@ -16131,7 +16131,7 @@
       </c>
       <c r="U150" t="inlineStr"/>
       <c r="V150" t="n">
-        <v>1.61</v>
+        <v>1.48</v>
       </c>
     </row>
     <row r="151">
@@ -16237,7 +16237,7 @@
       </c>
       <c r="U151" t="inlineStr"/>
       <c r="V151" t="n">
-        <v>1.88</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="152">
@@ -16343,7 +16343,7 @@
       </c>
       <c r="U152" t="inlineStr"/>
       <c r="V152" t="n">
-        <v>1.33</v>
+        <v>1.52</v>
       </c>
     </row>
     <row r="153">
@@ -16449,7 +16449,7 @@
       </c>
       <c r="U153" t="inlineStr"/>
       <c r="V153" t="n">
-        <v>1.31</v>
+        <v>1.82</v>
       </c>
     </row>
     <row r="154">
@@ -16555,7 +16555,7 @@
       </c>
       <c r="U154" t="inlineStr"/>
       <c r="V154" t="n">
-        <v>1.35</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="155">
@@ -16657,7 +16657,7 @@
       </c>
       <c r="U155" t="inlineStr"/>
       <c r="V155" t="n">
-        <v>1.54</v>
+        <v>1.46</v>
       </c>
     </row>
     <row r="156">
@@ -16763,7 +16763,7 @@
       </c>
       <c r="U156" t="inlineStr"/>
       <c r="V156" t="n">
-        <v>1.68</v>
+        <v>1.59</v>
       </c>
     </row>
     <row r="157">
@@ -16865,7 +16865,7 @@
       </c>
       <c r="U157" t="inlineStr"/>
       <c r="V157" t="n">
-        <v>1.64</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="158">
@@ -16971,7 +16971,7 @@
       </c>
       <c r="U158" t="inlineStr"/>
       <c r="V158" t="n">
-        <v>1.59</v>
+        <v>1.66</v>
       </c>
     </row>
     <row r="159">
@@ -17077,7 +17077,7 @@
       </c>
       <c r="U159" t="inlineStr"/>
       <c r="V159" t="n">
-        <v>1.73</v>
+        <v>1.76</v>
       </c>
     </row>
     <row r="160">
@@ -17183,7 +17183,7 @@
       </c>
       <c r="U160" t="inlineStr"/>
       <c r="V160" t="n">
-        <v>1.27</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="161">
@@ -17285,7 +17285,7 @@
       </c>
       <c r="U161" t="inlineStr"/>
       <c r="V161" t="n">
-        <v>1.74</v>
+        <v>1.18</v>
       </c>
     </row>
     <row r="162">
@@ -17391,7 +17391,7 @@
       </c>
       <c r="U162" t="inlineStr"/>
       <c r="V162" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="163">
@@ -17497,7 +17497,7 @@
       </c>
       <c r="U163" t="inlineStr"/>
       <c r="V163" t="n">
-        <v>1.67</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="164">
@@ -17603,7 +17603,7 @@
       </c>
       <c r="U164" t="inlineStr"/>
       <c r="V164" t="n">
-        <v>1.5</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="165">
@@ -17709,7 +17709,7 @@
       </c>
       <c r="U165" t="inlineStr"/>
       <c r="V165" t="n">
-        <v>1.29</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="166">
@@ -17815,7 +17815,7 @@
       </c>
       <c r="U166" t="inlineStr"/>
       <c r="V166" t="n">
-        <v>1.75</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="167">
@@ -17921,7 +17921,7 @@
       </c>
       <c r="U167" t="inlineStr"/>
       <c r="V167" t="n">
-        <v>1.41</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="168">
@@ -18027,7 +18027,7 @@
       </c>
       <c r="U168" t="inlineStr"/>
       <c r="V168" t="n">
-        <v>1.45</v>
+        <v>3.57</v>
       </c>
     </row>
     <row r="169">
@@ -18133,7 +18133,7 @@
       </c>
       <c r="U169" t="inlineStr"/>
       <c r="V169" t="n">
-        <v>1.25</v>
+        <v>3.76</v>
       </c>
     </row>
     <row r="170">
@@ -18239,7 +18239,7 @@
       </c>
       <c r="U170" t="inlineStr"/>
       <c r="V170" t="n">
-        <v>1.36</v>
+        <v>3.55</v>
       </c>
     </row>
     <row r="171">
@@ -18345,7 +18345,7 @@
       </c>
       <c r="U171" t="inlineStr"/>
       <c r="V171" t="n">
-        <v>1.99</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="172">
@@ -18447,7 +18447,7 @@
       </c>
       <c r="U172" t="inlineStr"/>
       <c r="V172" t="n">
-        <v>1.42</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="173">
@@ -18553,7 +18553,7 @@
       </c>
       <c r="U173" t="inlineStr"/>
       <c r="V173" t="n">
-        <v>2.84</v>
+        <v>1.61</v>
       </c>
     </row>
     <row r="174">
@@ -18659,7 +18659,7 @@
       </c>
       <c r="U174" t="inlineStr"/>
       <c r="V174" t="n">
-        <v>1.64</v>
+        <v>3.52</v>
       </c>
     </row>
     <row r="175">
@@ -18765,7 +18765,7 @@
       </c>
       <c r="U175" t="inlineStr"/>
       <c r="V175" t="n">
-        <v>1.7</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="176">
@@ -18871,7 +18871,7 @@
       </c>
       <c r="U176" t="inlineStr"/>
       <c r="V176" t="n">
-        <v>1.64</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="177">
@@ -18973,7 +18973,7 @@
       </c>
       <c r="U177" t="inlineStr"/>
       <c r="V177" t="n">
-        <v>1.47</v>
+        <v>2.44</v>
       </c>
     </row>
     <row r="178">
@@ -19075,7 +19075,7 @@
       </c>
       <c r="U178" t="inlineStr"/>
       <c r="V178" t="n">
-        <v>0.95</v>
+        <v>2.72</v>
       </c>
     </row>
     <row r="179">
@@ -19177,7 +19177,7 @@
       </c>
       <c r="U179" t="inlineStr"/>
       <c r="V179" t="n">
-        <v>1.67</v>
+        <v>2.93</v>
       </c>
     </row>
     <row r="180">
@@ -19283,7 +19283,7 @@
       </c>
       <c r="U180" t="inlineStr"/>
       <c r="V180" t="n">
-        <v>1.58</v>
+        <v>2.61</v>
       </c>
     </row>
     <row r="181">
@@ -19389,7 +19389,7 @@
       </c>
       <c r="U181" t="inlineStr"/>
       <c r="V181" t="n">
-        <v>3.93</v>
+        <v>1.97</v>
       </c>
     </row>
     <row r="182">
@@ -19491,7 +19491,7 @@
       </c>
       <c r="U182" t="inlineStr"/>
       <c r="V182" t="n">
-        <v>1.6</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="183">
@@ -19593,7 +19593,7 @@
       </c>
       <c r="U183" t="inlineStr"/>
       <c r="V183" t="n">
-        <v>1.45</v>
+        <v>4.04</v>
       </c>
     </row>
     <row r="184">
@@ -19699,7 +19699,7 @@
       </c>
       <c r="U184" t="inlineStr"/>
       <c r="V184" t="n">
-        <v>1.53</v>
+        <v>3.16</v>
       </c>
     </row>
     <row r="185">
@@ -19805,7 +19805,7 @@
       </c>
       <c r="U185" t="inlineStr"/>
       <c r="V185" t="n">
-        <v>1.53</v>
+        <v>4.35</v>
       </c>
     </row>
     <row r="186">
@@ -19911,7 +19911,7 @@
       </c>
       <c r="U186" t="inlineStr"/>
       <c r="V186" t="n">
-        <v>1.25</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="187">
@@ -20013,7 +20013,7 @@
       </c>
       <c r="U187" t="inlineStr"/>
       <c r="V187" t="n">
-        <v>1.47</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="188">
@@ -20119,7 +20119,7 @@
       </c>
       <c r="U188" t="inlineStr"/>
       <c r="V188" t="n">
-        <v>1.31</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="189">
@@ -20221,7 +20221,7 @@
       </c>
       <c r="U189" t="inlineStr"/>
       <c r="V189" t="n">
-        <v>1.64</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="190">
@@ -20327,7 +20327,7 @@
       </c>
       <c r="U190" t="inlineStr"/>
       <c r="V190" t="n">
-        <v>1.84</v>
+        <v>1.27</v>
       </c>
     </row>
     <row r="191">
@@ -20429,7 +20429,7 @@
       </c>
       <c r="U191" t="inlineStr"/>
       <c r="V191" t="n">
-        <v>1.09</v>
+        <v>5.56</v>
       </c>
     </row>
     <row r="192">
@@ -20531,7 +20531,7 @@
       </c>
       <c r="U192" t="inlineStr"/>
       <c r="V192" t="n">
-        <v>1.89</v>
+        <v>2.18</v>
       </c>
     </row>
     <row r="193">
@@ -20637,7 +20637,7 @@
       </c>
       <c r="U193" t="inlineStr"/>
       <c r="V193" t="n">
-        <v>1.99</v>
+        <v>7.91</v>
       </c>
     </row>
     <row r="194">
@@ -20739,7 +20739,7 @@
       </c>
       <c r="U194" t="inlineStr"/>
       <c r="V194" t="n">
-        <v>1.49</v>
+        <v>4.16</v>
       </c>
     </row>
     <row r="195">
@@ -20845,7 +20845,7 @@
       </c>
       <c r="U195" t="inlineStr"/>
       <c r="V195" t="n">
-        <v>1.31</v>
+        <v>3.81</v>
       </c>
     </row>
     <row r="196">
@@ -20951,7 +20951,7 @@
       </c>
       <c r="U196" t="inlineStr"/>
       <c r="V196" t="n">
-        <v>1.73</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="197">
@@ -21053,7 +21053,7 @@
       </c>
       <c r="U197" t="inlineStr"/>
       <c r="V197" t="n">
-        <v>1.57</v>
+        <v>1.34</v>
       </c>
     </row>
     <row r="198">
@@ -21159,7 +21159,7 @@
       </c>
       <c r="U198" t="inlineStr"/>
       <c r="V198" t="n">
-        <v>1.36</v>
+        <v>1.87</v>
       </c>
     </row>
     <row r="199">
@@ -21261,7 +21261,7 @@
       </c>
       <c r="U199" t="inlineStr"/>
       <c r="V199" t="n">
-        <v>1.48</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="200">
@@ -21363,7 +21363,7 @@
       </c>
       <c r="U200" t="inlineStr"/>
       <c r="V200" t="n">
-        <v>1.24</v>
+        <v>3.96</v>
       </c>
     </row>
     <row r="201">
@@ -21469,7 +21469,7 @@
       </c>
       <c r="U201" t="inlineStr"/>
       <c r="V201" t="n">
-        <v>2.83</v>
+        <v>2.54</v>
       </c>
     </row>
     <row r="202">
@@ -21575,7 +21575,7 @@
       </c>
       <c r="U202" t="inlineStr"/>
       <c r="V202" t="n">
-        <v>1.64</v>
+        <v>5.85</v>
       </c>
     </row>
     <row r="203">
@@ -21681,7 +21681,7 @@
       </c>
       <c r="U203" t="inlineStr"/>
       <c r="V203" t="n">
-        <v>1.69</v>
+        <v>5.02</v>
       </c>
     </row>
     <row r="204">
@@ -21787,7 +21787,7 @@
       </c>
       <c r="U204" t="inlineStr"/>
       <c r="V204" t="n">
-        <v>1.6</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="205">
@@ -21893,7 +21893,7 @@
       </c>
       <c r="U205" t="inlineStr"/>
       <c r="V205" t="n">
-        <v>2.24</v>
+        <v>3.58</v>
       </c>
     </row>
     <row r="206">
@@ -21995,7 +21995,7 @@
       </c>
       <c r="U206" t="inlineStr"/>
       <c r="V206" t="n">
-        <v>1.42</v>
+        <v>1.99</v>
       </c>
     </row>
     <row r="207">
@@ -22101,7 +22101,7 @@
       </c>
       <c r="U207" t="inlineStr"/>
       <c r="V207" t="n">
-        <v>1.6</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="208">
@@ -22207,7 +22207,7 @@
       </c>
       <c r="U208" t="inlineStr"/>
       <c r="V208" t="n">
-        <v>1.74</v>
+        <v>1.53</v>
       </c>
     </row>
     <row r="209">
@@ -22313,7 +22313,7 @@
       </c>
       <c r="U209" t="inlineStr"/>
       <c r="V209" t="n">
-        <v>1.78</v>
+        <v>1.69</v>
       </c>
     </row>
     <row r="210">
@@ -22415,7 +22415,7 @@
       </c>
       <c r="U210" t="inlineStr"/>
       <c r="V210" t="n">
-        <v>0.9399999999999999</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="211">
@@ -22521,7 +22521,7 @@
       </c>
       <c r="U211" t="inlineStr"/>
       <c r="V211" t="n">
-        <v>1.62</v>
+        <v>3.06</v>
       </c>
     </row>
     <row r="212">
@@ -22627,7 +22627,7 @@
       </c>
       <c r="U212" t="inlineStr"/>
       <c r="V212" t="n">
-        <v>1.3</v>
+        <v>2.94</v>
       </c>
     </row>
     <row r="213">
@@ -22733,7 +22733,7 @@
       </c>
       <c r="U213" t="inlineStr"/>
       <c r="V213" t="n">
-        <v>1.26</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="214">
@@ -22839,7 +22839,7 @@
       </c>
       <c r="U214" t="inlineStr"/>
       <c r="V214" t="n">
-        <v>1.29</v>
+        <v>2.32</v>
       </c>
     </row>
     <row r="215">
@@ -22945,7 +22945,7 @@
       </c>
       <c r="U215" t="inlineStr"/>
       <c r="V215" t="n">
-        <v>1.84</v>
+        <v>9.58</v>
       </c>
     </row>
     <row r="216">
@@ -23051,7 +23051,7 @@
       </c>
       <c r="U216" t="inlineStr"/>
       <c r="V216" t="n">
-        <v>1.97</v>
+        <v>4.51</v>
       </c>
     </row>
     <row r="217">
@@ -23157,7 +23157,7 @@
       </c>
       <c r="U217" t="inlineStr"/>
       <c r="V217" t="n">
-        <v>1.08</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="218">
@@ -23263,7 +23263,7 @@
       </c>
       <c r="U218" t="inlineStr"/>
       <c r="V218" t="n">
-        <v>1.6</v>
+        <v>4.26</v>
       </c>
     </row>
     <row r="219">
@@ -23369,7 +23369,7 @@
       </c>
       <c r="U219" t="inlineStr"/>
       <c r="V219" t="n">
-        <v>1.28</v>
+        <v>27.1</v>
       </c>
     </row>
     <row r="220">
@@ -23475,7 +23475,7 @@
       </c>
       <c r="U220" t="inlineStr"/>
       <c r="V220" t="n">
-        <v>1.54</v>
+        <v>43.42</v>
       </c>
     </row>
     <row r="221">
@@ -23581,7 +23581,7 @@
       </c>
       <c r="U221" t="inlineStr"/>
       <c r="V221" t="n">
-        <v>1.56</v>
+        <v>38.63</v>
       </c>
     </row>
     <row r="222">
@@ -23683,7 +23683,7 @@
       </c>
       <c r="U222" t="inlineStr"/>
       <c r="V222" t="n">
-        <v>2.15</v>
+        <v>38.9</v>
       </c>
     </row>
     <row r="223">
@@ -23789,7 +23789,7 @@
       </c>
       <c r="U223" t="inlineStr"/>
       <c r="V223" t="n">
-        <v>1.73</v>
+        <v>35.42</v>
       </c>
     </row>
     <row r="224">
@@ -23895,7 +23895,7 @@
       </c>
       <c r="U224" t="inlineStr"/>
       <c r="V224" t="n">
-        <v>1.58</v>
+        <v>25.28</v>
       </c>
     </row>
     <row r="225">
@@ -24001,7 +24001,7 @@
       </c>
       <c r="U225" t="inlineStr"/>
       <c r="V225" t="n">
-        <v>2.04</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="226">
@@ -24103,7 +24103,7 @@
       </c>
       <c r="U226" t="inlineStr"/>
       <c r="V226" t="n">
-        <v>1.56</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="227">
@@ -24209,7 +24209,7 @@
       </c>
       <c r="U227" t="inlineStr"/>
       <c r="V227" t="n">
-        <v>1.51</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="228">
@@ -24315,7 +24315,7 @@
       </c>
       <c r="U228" t="inlineStr"/>
       <c r="V228" t="n">
-        <v>1.44</v>
+        <v>2.07</v>
       </c>
     </row>
     <row r="229">
@@ -24417,7 +24417,7 @@
       </c>
       <c r="U229" t="inlineStr"/>
       <c r="V229" t="n">
-        <v>2.15</v>
+        <v>2.24</v>
       </c>
     </row>
     <row r="230">
@@ -24523,7 +24523,7 @@
       </c>
       <c r="U230" t="inlineStr"/>
       <c r="V230" t="n">
-        <v>1.6</v>
+        <v>3.02</v>
       </c>
     </row>
     <row r="231">
@@ -24625,7 +24625,7 @@
       </c>
       <c r="U231" t="inlineStr"/>
       <c r="V231" t="n">
-        <v>1.36</v>
+        <v>6.44</v>
       </c>
     </row>
     <row r="232">
@@ -24731,7 +24731,7 @@
       </c>
       <c r="U232" t="inlineStr"/>
       <c r="V232" t="n">
-        <v>1.41</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="233">
@@ -24833,7 +24833,7 @@
       </c>
       <c r="U233" t="inlineStr"/>
       <c r="V233" t="n">
-        <v>1.16</v>
+        <v>6.18</v>
       </c>
     </row>
     <row r="234">
@@ -24939,7 +24939,7 @@
       </c>
       <c r="U234" t="inlineStr"/>
       <c r="V234" t="n">
-        <v>1.24</v>
+        <v>5.19</v>
       </c>
     </row>
     <row r="235">
@@ -25041,7 +25041,7 @@
       </c>
       <c r="U235" t="inlineStr"/>
       <c r="V235" t="n">
-        <v>1.21</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="236">
@@ -25147,7 +25147,7 @@
       </c>
       <c r="U236" t="inlineStr"/>
       <c r="V236" t="n">
-        <v>1.84</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="237">
@@ -25249,7 +25249,7 @@
       </c>
       <c r="U237" t="inlineStr"/>
       <c r="V237" t="n">
-        <v>1.59</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="238">
@@ -25351,7 +25351,7 @@
       </c>
       <c r="U238" t="inlineStr"/>
       <c r="V238" t="n">
-        <v>3.16</v>
+        <v>2.64</v>
       </c>
     </row>
     <row r="239">
@@ -25457,7 +25457,7 @@
       </c>
       <c r="U239" t="inlineStr"/>
       <c r="V239" t="n">
-        <v>2.15</v>
+        <v>2.68</v>
       </c>
     </row>
     <row r="240">
@@ -25563,7 +25563,7 @@
       </c>
       <c r="U240" t="inlineStr"/>
       <c r="V240" t="n">
-        <v>3.1</v>
+        <v>2.79</v>
       </c>
     </row>
     <row r="241">
@@ -25669,7 +25669,7 @@
       </c>
       <c r="U241" t="inlineStr"/>
       <c r="V241" t="n">
-        <v>1.3</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="242">
@@ -25775,7 +25775,7 @@
       </c>
       <c r="U242" t="inlineStr"/>
       <c r="V242" t="n">
-        <v>1.31</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="243">
@@ -25877,7 +25877,7 @@
       </c>
       <c r="U243" t="inlineStr"/>
       <c r="V243" t="n">
-        <v>1.2</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="244">
@@ -25983,7 +25983,7 @@
       </c>
       <c r="U244" t="inlineStr"/>
       <c r="V244" t="n">
-        <v>1.64</v>
+        <v>1.17</v>
       </c>
     </row>
     <row r="245">
@@ -26089,7 +26089,7 @@
       </c>
       <c r="U245" t="inlineStr"/>
       <c r="V245" t="n">
-        <v>1.08</v>
+        <v>1.83</v>
       </c>
     </row>
     <row r="246">
@@ -26195,7 +26195,7 @@
       </c>
       <c r="U246" t="inlineStr"/>
       <c r="V246" t="n">
-        <v>1.55</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="247">
@@ -26297,7 +26297,7 @@
       </c>
       <c r="U247" t="inlineStr"/>
       <c r="V247" t="n">
-        <v>1.65</v>
+        <v>1.64</v>
       </c>
     </row>
     <row r="248">
@@ -26399,7 +26399,7 @@
       </c>
       <c r="U248" t="inlineStr"/>
       <c r="V248" t="n">
-        <v>1.34</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="249">
@@ -26505,7 +26505,7 @@
       </c>
       <c r="U249" t="inlineStr"/>
       <c r="V249" t="n">
-        <v>1.59</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="250">
@@ -26611,7 +26611,7 @@
       </c>
       <c r="U250" t="inlineStr"/>
       <c r="V250" t="n">
-        <v>1.77</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="251">
@@ -26717,7 +26717,7 @@
       </c>
       <c r="U251" t="inlineStr"/>
       <c r="V251" t="n">
-        <v>1.21</v>
+        <v>1.61</v>
       </c>
     </row>
     <row r="252">

</xml_diff>